<commit_message>
fix sheet to Data Manager schema
</commit_message>
<xml_diff>
--- a/stellar-conv/stellar-conv.xlsx
+++ b/stellar-conv/stellar-conv.xlsx
@@ -49,9 +49,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,63 +418,69 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Gbraid</t>
+          <t>Conversion action</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Conversion Name</t>
+          <t>GBRAID</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Conversion Time</t>
+          <t>Conversion date and time</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Conversion Value</t>
+          <t>Conversion value</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Conversion Currency</t>
+          <t>Conversion currency</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Order ID</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Conversion source</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>0AAAABDksRKwW_rAu0pt2xHebbnJ4X4yux</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-10-13 07:16:38-04:00</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T07:16:38-04:00</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -487,6 +494,11 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>187a50bc86824d0eb76824dd5cf3df7d</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Web</t>
         </is>
       </c>
     </row>

</xml_diff>